<commit_message>
updated excel ran convert.py all works
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D8E1390-2F75-B545-A7AE-99D7C7F700A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB864DD-AB27-4340-A790-8CDFA131F5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60160" yWindow="-3100" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="167">
   <si>
     <t>phase_id</t>
   </si>
@@ -98,7 +98,7 @@
     <t xml:space="preserve"> col-1</t>
   </si>
   <si>
-    <t xml:space="preserve"> cat-2</t>
+    <t>task-3</t>
   </si>
   <si>
     <t>phase_name</t>
@@ -330,6 +330,252 @@
 Höga höjder
 Etc.
 Teknisk chef</t>
+  </si>
+  <si>
+    <t>Rättigheterna bokade (spelrättigheter)</t>
+  </si>
+  <si>
+    <t>Preliminär budgetering</t>
+  </si>
+  <si>
+    <t>Arbetsfördelning</t>
+  </si>
+  <si>
+    <t>Vid behov börjar utredning för musikrättigheter
+Ansvarig dramaturg / Teaterchef</t>
+  </si>
+  <si>
+    <t>Hela organisationens budgeter
+Förvaltningschef
+Produktionsbudgeter
+Ansvarig producent
+Budgeterna skall anpassas med varandra</t>
+  </si>
+  <si>
+    <t>Fastanställda skådespelare
+Teaterchef, Ansvarig dramaturg, Ansvarig producent
+Fastanställda (interna) planerare
+Husets egen personal som gör planeringsuppdrag
+Teknisk chef, Ateljéchef, Teaterchef, Ansvarig dramaturg</t>
+  </si>
+  <si>
+    <t>task-4</t>
+  </si>
+  <si>
+    <t>task-5</t>
+  </si>
+  <si>
+    <t>task-6</t>
+  </si>
+  <si>
+    <t>task-7</t>
+  </si>
+  <si>
+    <t>task-8</t>
+  </si>
+  <si>
+    <t>task-9</t>
+  </si>
+  <si>
+    <t>task-10</t>
+  </si>
+  <si>
+    <t>task-11</t>
+  </si>
+  <si>
+    <t>task-12</t>
+  </si>
+  <si>
+    <t>task-13</t>
+  </si>
+  <si>
+    <t>task-14</t>
+  </si>
+  <si>
+    <t>task-15</t>
+  </si>
+  <si>
+    <t>task-16</t>
+  </si>
+  <si>
+    <t>task-17</t>
+  </si>
+  <si>
+    <t>task-18</t>
+  </si>
+  <si>
+    <t>task-19</t>
+  </si>
+  <si>
+    <t>task-20</t>
+  </si>
+  <si>
+    <t>task-21</t>
+  </si>
+  <si>
+    <t>task-22</t>
+  </si>
+  <si>
+    <t>task-23</t>
+  </si>
+  <si>
+    <t>task-24</t>
+  </si>
+  <si>
+    <t>task-25</t>
+  </si>
+  <si>
+    <t>task-26</t>
+  </si>
+  <si>
+    <t>task-27</t>
+  </si>
+  <si>
+    <t>task-28</t>
+  </si>
+  <si>
+    <t>task-29</t>
+  </si>
+  <si>
+    <t>task-30</t>
+  </si>
+  <si>
+    <t>task-31</t>
+  </si>
+  <si>
+    <t>task-32</t>
+  </si>
+  <si>
+    <t>task-33</t>
+  </si>
+  <si>
+    <t>task-34</t>
+  </si>
+  <si>
+    <t>task-35</t>
+  </si>
+  <si>
+    <t>task-36</t>
+  </si>
+  <si>
+    <t>task-37</t>
+  </si>
+  <si>
+    <t>task-38</t>
+  </si>
+  <si>
+    <t>task-39</t>
+  </si>
+  <si>
+    <t>task-40</t>
+  </si>
+  <si>
+    <t>task-41</t>
+  </si>
+  <si>
+    <t>task-42</t>
+  </si>
+  <si>
+    <t>task-43</t>
+  </si>
+  <si>
+    <t>task-44</t>
+  </si>
+  <si>
+    <t>task-45</t>
+  </si>
+  <si>
+    <t>task-46</t>
+  </si>
+  <si>
+    <t>Ljud</t>
+  </si>
+  <si>
+    <t>Ljus</t>
+  </si>
+  <si>
+    <t>Rekvisita</t>
+  </si>
+  <si>
+    <t>Pyro</t>
+  </si>
+  <si>
+    <t>Video</t>
+  </si>
+  <si>
+    <t>Kostym</t>
+  </si>
+  <si>
+    <t>Mask &amp; hår</t>
+  </si>
+  <si>
+    <t>Utrymmen</t>
+  </si>
+  <si>
+    <t>Musik</t>
+  </si>
+  <si>
+    <t>Förslag på regissör</t>
+  </si>
+  <si>
+    <t>Regissören vald</t>
+  </si>
+  <si>
+    <t>Manuskript, v. 1</t>
+  </si>
+  <si>
+    <t>Antal skådespelare, antal roller, barn, djur etc</t>
+  </si>
+  <si>
+    <t>Personalresursering</t>
+  </si>
+  <si>
+    <t>Textning</t>
+  </si>
+  <si>
+    <t>Försäljningsprognos</t>
+  </si>
+  <si>
+    <t>Specialmålgrupper</t>
+  </si>
+  <si>
+    <t>Beslut Premiär / Presspremiär</t>
+  </si>
+  <si>
+    <t>Statistik</t>
+  </si>
+  <si>
+    <t>Projektkod</t>
+  </si>
+  <si>
+    <t>Slotifiering färdig</t>
+  </si>
+  <si>
+    <t>Turné/byte av scen</t>
+  </si>
+  <si>
+    <t>Teaterns beställning av regissören</t>
+  </si>
+  <si>
+    <t>Repetitionsplanering</t>
+  </si>
+  <si>
+    <t>Produktionsbeslut DL</t>
+  </si>
+  <si>
+    <t>Porttidtabell</t>
+  </si>
+  <si>
+    <t>Rättigheterna förhandlade</t>
+  </si>
+  <si>
+    <t>Preliminärt produktionsberedingsdokument</t>
+  </si>
+  <si>
+    <t>Toimintasuunnitelma kolmelle vuodelle</t>
+  </si>
+  <si>
+    <t>Teknisk beredskap</t>
   </si>
 </sst>
 </file>
@@ -924,12 +1170,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D990BC4-CB70-7945-A3FE-EC48E23980DB}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -955,7 +1201,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="404" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="340" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -965,7 +1211,7 @@
       <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -975,27 +1221,638 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>115</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
         <v>18</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E27" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
+      <c r="G27" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" t="s">
+        <v>18</v>
+      </c>
+      <c r="E29" t="s">
+        <v>138</v>
+      </c>
+      <c r="G29" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" t="s">
+        <v>139</v>
+      </c>
+      <c r="G30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+      <c r="E31" t="s">
+        <v>140</v>
+      </c>
+      <c r="G31" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" t="s">
+        <v>141</v>
+      </c>
+      <c r="G32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" t="s">
+        <v>18</v>
+      </c>
+      <c r="E33" t="s">
+        <v>142</v>
+      </c>
+      <c r="G33" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>123</v>
+      </c>
+      <c r="B34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" t="s">
+        <v>143</v>
+      </c>
+      <c r="G34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="E35" t="s">
+        <v>144</v>
+      </c>
+      <c r="G35" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>125</v>
+      </c>
+      <c r="B36" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" t="s">
+        <v>74</v>
+      </c>
+      <c r="G36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" t="s">
+        <v>145</v>
+      </c>
+      <c r="G37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>129</v>
+      </c>
+      <c r="B40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>130</v>
+      </c>
+      <c r="B41" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>131</v>
+      </c>
+      <c r="B42" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>132</v>
+      </c>
+      <c r="B43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>133</v>
+      </c>
+      <c r="B44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>135</v>
+      </c>
+      <c r="B46" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E49" s="2"/>
+      <c r="F49" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
more data, still vertical
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB864DD-AB27-4340-A790-8CDFA131F5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8581684B-09CF-F04B-A9BD-BF9FF9744344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60160" yWindow="-3100" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
+    <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Faser" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="283">
   <si>
     <t>phase_id</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve"> phase-1</t>
+  </si>
+  <si>
+    <t>col-2</t>
   </si>
   <si>
     <t>task_id</t>
@@ -317,9 +320,6 @@
     <t xml:space="preserve"> task_title</t>
   </si>
   <si>
-    <t xml:space="preserve"> phase-3</t>
-  </si>
-  <si>
     <t>Scenografi</t>
   </si>
   <si>
@@ -576,6 +576,357 @@
   </si>
   <si>
     <t>Teknisk beredskap</t>
+  </si>
+  <si>
+    <t>Rättigheternas avtal undertecknade</t>
+  </si>
+  <si>
+    <t>Manuskript på svenska</t>
+  </si>
+  <si>
+    <t>Val av konstnärliga teamet + kontrakt</t>
+  </si>
+  <si>
+    <t>Kartläggning av produktionens datum</t>
+  </si>
+  <si>
+    <t>Produktionsbudget</t>
+  </si>
+  <si>
+    <t>Planerarnas kontrakt</t>
+  </si>
+  <si>
+    <t>Theatron</t>
+  </si>
+  <si>
+    <t>Intern definition av tekniska ramar</t>
+  </si>
+  <si>
+    <t>Preliminär ramdiskussion (TÄMÄ TURHA?)</t>
+  </si>
+  <si>
+    <t>Ramarnas kommunicering till konstnärliga teamet</t>
+  </si>
+  <si>
+    <t>Personalresursering tekniken</t>
+  </si>
+  <si>
+    <t>Scenografi &gt; Teknisk chef</t>
+  </si>
+  <si>
+    <t>Stora scenen</t>
+  </si>
+  <si>
+    <t>Amos</t>
+  </si>
+  <si>
+    <t>Nicken</t>
+  </si>
+  <si>
+    <t>Ljud &gt; Teknisk chef</t>
+  </si>
+  <si>
+    <t>Ljus &amp; Video &gt; Teknisk chef</t>
+  </si>
+  <si>
+    <t>Ateljéchef</t>
+  </si>
+  <si>
+    <t>Teaterchef</t>
+  </si>
+  <si>
+    <t>produktionens behov diskuteras i förhållande till resurserna och övriga produktioner (teknisk förhandsplanering)</t>
+  </si>
+  <si>
+    <t>Mask</t>
+  </si>
+  <si>
+    <t>Koreograf</t>
+  </si>
+  <si>
+    <t>Kapellmästare</t>
+  </si>
+  <si>
+    <t>Orkesterplacering</t>
+  </si>
+  <si>
+    <t>Behov av regiassistent</t>
+  </si>
+  <si>
+    <t>Beslut om workshop</t>
+  </si>
+  <si>
+    <t>task-47</t>
+  </si>
+  <si>
+    <t>task-48</t>
+  </si>
+  <si>
+    <t>task-49</t>
+  </si>
+  <si>
+    <t>task-50</t>
+  </si>
+  <si>
+    <t>task-51</t>
+  </si>
+  <si>
+    <t>task-52</t>
+  </si>
+  <si>
+    <t>task-53</t>
+  </si>
+  <si>
+    <t>task-54</t>
+  </si>
+  <si>
+    <t>task-55</t>
+  </si>
+  <si>
+    <t>task-56</t>
+  </si>
+  <si>
+    <t>task-57</t>
+  </si>
+  <si>
+    <t>task-58</t>
+  </si>
+  <si>
+    <t>task-59</t>
+  </si>
+  <si>
+    <t>task-60</t>
+  </si>
+  <si>
+    <t>task-61</t>
+  </si>
+  <si>
+    <t>col-3</t>
+  </si>
+  <si>
+    <t>Teknisk chef</t>
+  </si>
+  <si>
+    <t>task-62</t>
+  </si>
+  <si>
+    <t>Verkstäder</t>
+  </si>
+  <si>
+    <t>Påklädare</t>
+  </si>
+  <si>
+    <t>task-63</t>
+  </si>
+  <si>
+    <t>task-64</t>
+  </si>
+  <si>
+    <t>task-65</t>
+  </si>
+  <si>
+    <t>task-66</t>
+  </si>
+  <si>
+    <t>task-67</t>
+  </si>
+  <si>
+    <t>task-68</t>
+  </si>
+  <si>
+    <t>task-69</t>
+  </si>
+  <si>
+    <t>task-70</t>
+  </si>
+  <si>
+    <t>Informationsmöte
+Ansvarig producent sammankallar
+Konstnärliga teamet, teknisk chef, ateljéchef, teaterchef, ansvarig dramaturg/föreställningsdramaturg, fm-chef, scenmästare, inspicient, teknisk planerare, informatör
+Produktionens ramar presenteras och fastslås</t>
+  </si>
+  <si>
+    <t>Planerarmöte (husets representanter på plats)</t>
+  </si>
+  <si>
+    <t>Reality check innan idémöte</t>
+  </si>
+  <si>
+    <t>Idémöte</t>
+  </si>
+  <si>
+    <t>task-71</t>
+  </si>
+  <si>
+    <t>task-72</t>
+  </si>
+  <si>
+    <t>task-73</t>
+  </si>
+  <si>
+    <t>Klassificering av rollerna (A/B)</t>
+  </si>
+  <si>
+    <t>Rollsättning, mått, namn</t>
+  </si>
+  <si>
+    <t>Casting klar</t>
+  </si>
+  <si>
+    <t>Försäljning &amp; Marknadsföring, Planering</t>
+  </si>
+  <si>
+    <t>Info till fasta skådespelare om kommande roller</t>
+  </si>
+  <si>
+    <t>Freelance-skådespelarnas kontrakt</t>
+  </si>
+  <si>
+    <t>LL-planerarträffar</t>
+  </si>
+  <si>
+    <t>Scenografiträffar</t>
+  </si>
+  <si>
+    <t>IT • HR-info</t>
+  </si>
+  <si>
+    <t>task-74</t>
+  </si>
+  <si>
+    <t>task-75</t>
+  </si>
+  <si>
+    <t>task-76</t>
+  </si>
+  <si>
+    <t>task-77</t>
+  </si>
+  <si>
+    <t>task-78</t>
+  </si>
+  <si>
+    <t>task-79</t>
+  </si>
+  <si>
+    <t>task-80</t>
+  </si>
+  <si>
+    <t>task-81</t>
+  </si>
+  <si>
+    <t>task-82</t>
+  </si>
+  <si>
+    <t>Preliminära modellens feedback</t>
+  </si>
+  <si>
+    <t>Föreställningsplan</t>
+  </si>
+  <si>
+    <t>Frilansteknikernas kontrakt (ÄR DENNA FÖR TIDIG?)</t>
+  </si>
+  <si>
+    <t>Modellens godkännande</t>
+  </si>
+  <si>
+    <t>Teknisk planering börjar</t>
+  </si>
+  <si>
+    <t>Modellens korrigering</t>
+  </si>
+  <si>
+    <t>Behov för 3D-ritningar</t>
+  </si>
+  <si>
+    <t>Preliminära ljud- och ljusplaner</t>
+  </si>
+  <si>
+    <t>Workshops / första läsning (ÄR DENNA FÖR SENT?)</t>
+  </si>
+  <si>
+    <t>obs</t>
+  </si>
+  <si>
+    <t>shelf</t>
+  </si>
+  <si>
+    <t>Planen för publikarbete</t>
+  </si>
+  <si>
+    <t>Kostymplanering klar</t>
+  </si>
+  <si>
+    <t>Maskplanering klar</t>
+  </si>
+  <si>
+    <t>Repetitioner – när och var?</t>
+  </si>
+  <si>
+    <t>Spelplan</t>
+  </si>
+  <si>
+    <t>Visumöte</t>
+  </si>
+  <si>
+    <t>Detaljerade FM-planer och materialproduktion</t>
+  </si>
+  <si>
+    <t>Lansering • förköpskampanjer</t>
+  </si>
+  <si>
+    <t>task-83</t>
+  </si>
+  <si>
+    <t>task-84</t>
+  </si>
+  <si>
+    <t>task-85</t>
+  </si>
+  <si>
+    <t>task-86</t>
+  </si>
+  <si>
+    <t>task-87</t>
+  </si>
+  <si>
+    <t>task-88</t>
+  </si>
+  <si>
+    <t>task-89</t>
+  </si>
+  <si>
+    <t>task-90</t>
+  </si>
+  <si>
+    <t>task-91</t>
+  </si>
+  <si>
+    <t>task-92</t>
+  </si>
+  <si>
+    <t>task-93</t>
+  </si>
+  <si>
+    <t>task-94</t>
+  </si>
+  <si>
+    <t>task-95</t>
+  </si>
+  <si>
+    <t>task-96</t>
+  </si>
+  <si>
+    <t>task-97</t>
+  </si>
+  <si>
+    <t>task-98</t>
+  </si>
+  <si>
+    <t>task-99</t>
+  </si>
+  <si>
+    <t>task-100</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -1005,7 +1356,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -1013,10 +1364,10 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1024,13 +1375,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
@@ -1038,128 +1389,131 @@
     </row>
     <row r="4" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1170,7 +1524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D990BC4-CB70-7945-A3FE-EC48E23980DB}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -1178,52 +1532,55 @@
     <col min="6" max="6" width="47.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="340" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="340" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -1235,12 +1592,12 @@
         <v>91</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -1252,10 +1609,10 @@
         <v>92</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1269,10 +1626,10 @@
         <v>93</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -1283,10 +1640,10 @@
         <v>157</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1297,10 +1654,10 @@
         <v>158</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -1311,10 +1668,10 @@
         <v>159</v>
       </c>
       <c r="G8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -1325,10 +1682,10 @@
         <v>160</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>99</v>
       </c>
@@ -1339,10 +1696,10 @@
         <v>161</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>100</v>
       </c>
@@ -1353,10 +1710,10 @@
         <v>162</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -1367,10 +1724,10 @@
         <v>163</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>102</v>
       </c>
@@ -1381,10 +1738,10 @@
         <v>164</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>103</v>
       </c>
@@ -1395,10 +1752,10 @@
         <v>165</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>104</v>
       </c>
@@ -1409,21 +1766,21 @@
         <v>166</v>
       </c>
       <c r="G15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>146</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1431,7 +1788,7 @@
         <v>106</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s">
         <v>105</v>
@@ -1440,7 +1797,7 @@
         <v>147</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1448,13 +1805,13 @@
         <v>107</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>148</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1462,13 +1819,13 @@
         <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>149</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1476,13 +1833,13 @@
         <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>150</v>
       </c>
       <c r="G20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1490,13 +1847,13 @@
         <v>110</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>151</v>
       </c>
       <c r="G21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1504,13 +1861,13 @@
         <v>111</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>152</v>
       </c>
       <c r="G22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1518,13 +1875,13 @@
         <v>112</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>153</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1532,13 +1889,13 @@
         <v>113</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>154</v>
       </c>
       <c r="G24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1546,13 +1903,13 @@
         <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>155</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1560,13 +1917,13 @@
         <v>115</v>
       </c>
       <c r="B26" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>156</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="136" x14ac:dyDescent="0.2">
@@ -1574,10 +1931,10 @@
         <v>116</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>86</v>
@@ -1586,7 +1943,7 @@
         <v>87</v>
       </c>
       <c r="G27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1594,16 +1951,16 @@
         <v>117</v>
       </c>
       <c r="B28" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C28" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>137</v>
       </c>
       <c r="G28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1611,16 +1968,16 @@
         <v>118</v>
       </c>
       <c r="B29" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>18</v>
-      </c>
-      <c r="E29" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>138</v>
       </c>
       <c r="G29" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1628,16 +1985,16 @@
         <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C30" t="s">
-        <v>18</v>
-      </c>
-      <c r="E30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>139</v>
       </c>
       <c r="G30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1645,16 +2002,16 @@
         <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s">
-        <v>18</v>
-      </c>
-      <c r="E31" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>140</v>
       </c>
       <c r="G31" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1662,194 +2019,1158 @@
         <v>121</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
-      </c>
-      <c r="E32" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>141</v>
       </c>
       <c r="G32" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>122</v>
       </c>
       <c r="B33" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
-      </c>
-      <c r="E33" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>142</v>
       </c>
       <c r="G33" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>123</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C34" t="s">
-        <v>18</v>
-      </c>
-      <c r="E34" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>143</v>
       </c>
       <c r="G34" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>124</v>
       </c>
       <c r="B35" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
-      </c>
-      <c r="E35" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>144</v>
       </c>
       <c r="G35" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>125</v>
       </c>
       <c r="B36" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C36" t="s">
-        <v>18</v>
-      </c>
-      <c r="E36" t="s">
-        <v>74</v>
+        <v>19</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="G36" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>126</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
-      </c>
-      <c r="E37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>145</v>
       </c>
       <c r="G37" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>127</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
-      </c>
-      <c r="C38" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G38" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>128</v>
       </c>
       <c r="B39" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G39" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>129</v>
       </c>
       <c r="B40" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G40" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>130</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G41" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>131</v>
       </c>
       <c r="B42" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G42" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>132</v>
       </c>
       <c r="B43" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G43" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>133</v>
       </c>
       <c r="B44" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G44" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>134</v>
       </c>
       <c r="B45" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G45" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>135</v>
       </c>
       <c r="B46" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G46" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>136</v>
       </c>
       <c r="B47" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+      <c r="C47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G47" t="s">
+        <v>63</v>
+      </c>
+      <c r="H47" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>193</v>
+      </c>
       <c r="B48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="49" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E49" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="C48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G48" t="s">
+        <v>63</v>
+      </c>
+      <c r="H48" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>194</v>
+      </c>
+      <c r="B49" t="s">
+        <v>28</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>181</v>
+      </c>
       <c r="F49" s="1"/>
+      <c r="G49" t="s">
+        <v>63</v>
+      </c>
+      <c r="H49" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>195</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G50" t="s">
+        <v>63</v>
+      </c>
+      <c r="H50" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>196</v>
+      </c>
+      <c r="B51" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G51" t="s">
+        <v>63</v>
+      </c>
+      <c r="H51" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>197</v>
+      </c>
+      <c r="B52" t="s">
+        <v>28</v>
+      </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G52" t="s">
+        <v>63</v>
+      </c>
+      <c r="H52" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>198</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G53" t="s">
+        <v>63</v>
+      </c>
+      <c r="H53" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>199</v>
+      </c>
+      <c r="B54" t="s">
+        <v>28</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G54" t="s">
+        <v>63</v>
+      </c>
+      <c r="H54" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B55" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G55" t="s">
+        <v>63</v>
+      </c>
+      <c r="H55" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>201</v>
+      </c>
+      <c r="B56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G56" t="s">
+        <v>68</v>
+      </c>
+      <c r="H56" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>202</v>
+      </c>
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G57" t="s">
+        <v>68</v>
+      </c>
+      <c r="H57" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>203</v>
+      </c>
+      <c r="B58" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G58" t="s">
+        <v>62</v>
+      </c>
+      <c r="H58" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>204</v>
+      </c>
+      <c r="B59" t="s">
+        <v>28</v>
+      </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G59" t="s">
+        <v>62</v>
+      </c>
+      <c r="H59" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>205</v>
+      </c>
+      <c r="B60" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G60" t="s">
+        <v>62</v>
+      </c>
+      <c r="H60" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>206</v>
+      </c>
+      <c r="B61" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G61" t="s">
+        <v>62</v>
+      </c>
+      <c r="H61" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>207</v>
+      </c>
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G62" t="s">
+        <v>62</v>
+      </c>
+      <c r="H62" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" t="s">
+        <v>208</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G63" t="s">
+        <v>62</v>
+      </c>
+      <c r="H63" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>213</v>
+      </c>
+      <c r="B64" t="s">
+        <v>28</v>
+      </c>
+      <c r="C64" t="s">
+        <v>208</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G64" t="s">
+        <v>62</v>
+      </c>
+      <c r="H64" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>214</v>
+      </c>
+      <c r="B65" t="s">
+        <v>28</v>
+      </c>
+      <c r="C65" t="s">
+        <v>208</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G65" t="s">
+        <v>62</v>
+      </c>
+      <c r="H65" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>215</v>
+      </c>
+      <c r="B66" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66" t="s">
+        <v>208</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G66" t="s">
+        <v>62</v>
+      </c>
+      <c r="H66" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>216</v>
+      </c>
+      <c r="B67" t="s">
+        <v>28</v>
+      </c>
+      <c r="C67" t="s">
+        <v>208</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G67" t="s">
+        <v>62</v>
+      </c>
+      <c r="H67" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>217</v>
+      </c>
+      <c r="B68" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68" t="s">
+        <v>208</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G68" t="s">
+        <v>62</v>
+      </c>
+      <c r="H68" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>218</v>
+      </c>
+      <c r="B69" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" t="s">
+        <v>208</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G69" t="s">
+        <v>68</v>
+      </c>
+      <c r="H69" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>219</v>
+      </c>
+      <c r="B70" t="s">
+        <v>28</v>
+      </c>
+      <c r="C70" t="s">
+        <v>208</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G70" t="s">
+        <v>68</v>
+      </c>
+      <c r="H70" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>220</v>
+      </c>
+      <c r="B71" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71" t="s">
+        <v>208</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G71" t="s">
+        <v>68</v>
+      </c>
+      <c r="H71" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>225</v>
+      </c>
+      <c r="B72" t="s">
+        <v>29</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G72" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>226</v>
+      </c>
+      <c r="B73" t="s">
+        <v>29</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G73" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>227</v>
+      </c>
+      <c r="B74" t="s">
+        <v>29</v>
+      </c>
+      <c r="D74" t="s">
+        <v>226</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G74" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>237</v>
+      </c>
+      <c r="B75" t="s">
+        <v>29</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G75" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>238</v>
+      </c>
+      <c r="B76" t="s">
+        <v>29</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G76" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>239</v>
+      </c>
+      <c r="B77" t="s">
+        <v>29</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>240</v>
+      </c>
+      <c r="B78" t="s">
+        <v>29</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G78" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>241</v>
+      </c>
+      <c r="B79" t="s">
+        <v>29</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G79" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>242</v>
+      </c>
+      <c r="B80" t="s">
+        <v>29</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G80" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>243</v>
+      </c>
+      <c r="B81" t="s">
+        <v>29</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G81" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>244</v>
+      </c>
+      <c r="B82" t="s">
+        <v>29</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G82" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>245</v>
+      </c>
+      <c r="B83" t="s">
+        <v>29</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G83" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>265</v>
+      </c>
+      <c r="B84" t="s">
+        <v>30</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G84" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>266</v>
+      </c>
+      <c r="B85" t="s">
+        <v>30</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G85" t="s">
+        <v>64</v>
+      </c>
+      <c r="H85" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>267</v>
+      </c>
+      <c r="B86" t="s">
+        <v>30</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G86" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>268</v>
+      </c>
+      <c r="B87" t="s">
+        <v>30</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G87" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>269</v>
+      </c>
+      <c r="B88" t="s">
+        <v>30</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G88" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>270</v>
+      </c>
+      <c r="B89" t="s">
+        <v>30</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G89" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>271</v>
+      </c>
+      <c r="B90" t="s">
+        <v>30</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="G90" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>272</v>
+      </c>
+      <c r="B91" t="s">
+        <v>30</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G91" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>273</v>
+      </c>
+      <c r="B92" t="s">
+        <v>30</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G92" t="s">
+        <v>72</v>
+      </c>
+      <c r="H92" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>274</v>
+      </c>
+      <c r="B93" t="s">
+        <v>30</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G93" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>275</v>
+      </c>
+      <c r="B94" t="s">
+        <v>30</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G94" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>276</v>
+      </c>
+      <c r="B95" t="s">
+        <v>30</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G95" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>277</v>
+      </c>
+      <c r="B96" t="s">
+        <v>30</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="G96" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>278</v>
+      </c>
+      <c r="B97" t="s">
+        <v>30</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="G97" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>279</v>
+      </c>
+      <c r="B98" t="s">
+        <v>30</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G98" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>280</v>
+      </c>
+      <c r="B99" t="s">
+        <v>30</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="G99" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>281</v>
+      </c>
+      <c r="B100" t="s">
+        <v>30</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G100" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>282</v>
+      </c>
+      <c r="B101" t="s">
+        <v>30</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G101" t="s">
+        <v>73</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1859,12 +3180,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F37668F2-ED8B-F149-837A-2B09ADA68CAE}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1876,10 +3197,10 @@
         <v>8</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="119" x14ac:dyDescent="0.2">
@@ -1887,13 +3208,38 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -1912,74 +3258,74 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vertical before duration_num data
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8581684B-09CF-F04B-A9BD-BF9FF9744344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EAB77B-9D7D-EC4D-8FDC-CE1CD65CDE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
+    <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Faser" sheetId="4" r:id="rId1"/>
@@ -39,12 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="285">
   <si>
     <t>phase_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> duration</t>
   </si>
   <si>
     <t xml:space="preserve"> port_title</t>
@@ -927,6 +924,15 @@
   </si>
   <si>
     <t>task-100</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>3,5,10</t>
+  </si>
+  <si>
+    <t>duration_num</t>
   </si>
 </sst>
 </file>
@@ -1329,191 +1335,224 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{844AD846-CE82-7641-9E59-3A5898370BA8}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.5" customWidth="1"/>
-    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.6640625" customWidth="1"/>
+    <col min="3" max="4" width="16.5" customWidth="1"/>
+    <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>283</v>
+      </c>
+      <c r="E9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="68" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
         <v>33</v>
       </c>
-      <c r="C4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="153" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="136" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="B12" s="2" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1524,7 +1563,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D990BC4-CB70-7945-A3FE-EC48E23980DB}">
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -1534,1642 +1573,1647 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="340" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G2" t="s">
         <v>16</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="136" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E27" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="G27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B39" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B41" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B43" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B44" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B45" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G45" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B46" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G46" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G47" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H47" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B48" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G48" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H48" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B49" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B50" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G50" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H50" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H51" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B52" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G52" t="s">
+        <v>62</v>
+      </c>
+      <c r="H52" t="s">
         <v>181</v>
-      </c>
-      <c r="G52" t="s">
-        <v>63</v>
-      </c>
-      <c r="H52" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B53" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G53" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H53" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B54" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H54" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H55" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B56" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G56" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H56" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B57" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G57" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H57" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B58" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H58" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B59" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G59" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H59" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B60" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H60" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H61" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G62" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
+        <v>209</v>
+      </c>
+      <c r="B63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C63" t="s">
+        <v>207</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B63" t="s">
-        <v>28</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="G63" t="s">
+        <v>61</v>
+      </c>
+      <c r="H63" t="s">
         <v>208</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="G63" t="s">
-        <v>62</v>
-      </c>
-      <c r="H63" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B64" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C64" t="s">
+        <v>207</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G64" t="s">
+        <v>61</v>
+      </c>
+      <c r="H64" t="s">
         <v>208</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G64" t="s">
-        <v>62</v>
-      </c>
-      <c r="H64" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C65" t="s">
+        <v>207</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G65" t="s">
+        <v>61</v>
+      </c>
+      <c r="H65" t="s">
         <v>208</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G65" t="s">
-        <v>62</v>
-      </c>
-      <c r="H65" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B66" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C66" t="s">
+        <v>207</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G66" t="s">
+        <v>61</v>
+      </c>
+      <c r="H66" t="s">
         <v>208</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="G66" t="s">
-        <v>62</v>
-      </c>
-      <c r="H66" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B67" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C67" t="s">
+        <v>207</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G67" t="s">
+        <v>61</v>
+      </c>
+      <c r="H67" t="s">
         <v>208</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G67" t="s">
-        <v>62</v>
-      </c>
-      <c r="H67" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B68" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C68" t="s">
+        <v>207</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G68" t="s">
+        <v>61</v>
+      </c>
+      <c r="H68" t="s">
         <v>208</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G68" t="s">
-        <v>62</v>
-      </c>
-      <c r="H68" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B69" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C69" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H69" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B70" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C70" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G70" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H70" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B71" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C71" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G71" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H71" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B72" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G72" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B73" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G73" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B74" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D74" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G74" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B75" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B76" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G76" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B77" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G77" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G78" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G79" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G80" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B81" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G81" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B82" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G82" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G83" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G84" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B85" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G85" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H85" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B86" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G86" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B87" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G87" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B88" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G88" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B89" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G89" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G90" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B91" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G91" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B92" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E92" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="G92" t="s">
+        <v>71</v>
+      </c>
+      <c r="H92" t="s">
         <v>254</v>
-      </c>
-      <c r="G92" t="s">
-        <v>72</v>
-      </c>
-      <c r="H92" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B93" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G93" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B94" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G94" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B95" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G95" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B96" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G96" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B97" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G97" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B98" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G98" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B99" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G99" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B100" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G100" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B101" t="s">
+        <v>29</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G101" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B102" t="s">
         <v>30</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="G101" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -3191,55 +3235,55 @@
   <sheetData>
     <row r="1" spans="1:4" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>8</v>
-      </c>
       <c r="C1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="119" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -3258,74 +3302,74 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
         <v>68</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
timeline length visualised prod date entered
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EAB77B-9D7D-EC4D-8FDC-CE1CD65CDE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6388662F-BCFE-174B-B3C5-1324176A13C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="313">
   <si>
     <t>phase_id</t>
   </si>
@@ -933,6 +933,104 @@
   </si>
   <si>
     <t>duration_num</t>
+  </si>
+  <si>
+    <t>Ritningar</t>
+  </si>
+  <si>
+    <t>Beställning av 3D-ritningar</t>
+  </si>
+  <si>
+    <t>Rekvisita startmöte</t>
+  </si>
+  <si>
+    <t>Scenbilder</t>
+  </si>
+  <si>
+    <t>Ljusplans uppföljning</t>
+  </si>
+  <si>
+    <t>Ljudplan uppföljning</t>
+  </si>
+  <si>
+    <t>Pyro / SFX plan</t>
+  </si>
+  <si>
+    <t>Repetitionsrekvisita</t>
+  </si>
+  <si>
+    <t>Anskaffningar</t>
+  </si>
+  <si>
+    <t>Tillverkning</t>
+  </si>
+  <si>
+    <t>Ateljé startmöten</t>
+  </si>
+  <si>
+    <t>Första kostymprovningar</t>
+  </si>
+  <si>
+    <t>Loger</t>
+  </si>
+  <si>
+    <t>Repetitionsplan</t>
+  </si>
+  <si>
+    <t>Produktionsmöten börjar</t>
+  </si>
+  <si>
+    <t>Frilansteknikernas kontrakt</t>
+  </si>
+  <si>
+    <t>obs - fanns i ett tidigare skede</t>
+  </si>
+  <si>
+    <t>Detaljerad rep.plan</t>
+  </si>
+  <si>
+    <t>Repstart check</t>
+  </si>
+  <si>
+    <t>Repstart mail till casten</t>
+  </si>
+  <si>
+    <t>Workshop</t>
+  </si>
+  <si>
+    <t>HR och IT</t>
+  </si>
+  <si>
+    <t>"När är det på riktigt taru, 10 dagar?"</t>
+  </si>
+  <si>
+    <t>Rep. Manus</t>
+  </si>
+  <si>
+    <t>Publikarbetets plan</t>
+  </si>
+  <si>
+    <t>Taktiska marknadsföringsåtgärder</t>
+  </si>
+  <si>
+    <t>Ansvarig producent sammankallar
+Informationsmöte
+Tekniska chefen och Ateljéchefen agerar ordförande
+Ansvarig producent agerar sekreterare
+Närvarande: Teknisk chef, Ateljéchef, Ansvarig producent, Teknisk planerare, konstnärliga teamet 
+Öppet till alla i huset
+Datumet informeras om i prod.rådet</t>
+  </si>
+  <si>
+    <t>Ansvarig producent sammankallar
+Diskussionsmöte
+Ansvarig producent, Teknisk chef, Ateljéchef, Scenograf, Teknisk planerare, Kläddesigner, övriga konstnärliga teamet frivilligt
+Teknisk chef och Ateljéchef agerar ordförande
+Ansvarig producent agerar sekreterare
+De ansvariga planerarna presenterar de preliminära planerna för:
+Scenografi
+Kostym
+Övriga vid behov</t>
   </si>
 </sst>
 </file>
@@ -1462,7 +1560,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="204" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1478,8 +1576,11 @@
       <c r="E7" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G7" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="136" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1494,6 +1595,9 @@
       </c>
       <c r="E8" t="s">
         <v>47</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1563,7 +1667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D990BC4-CB70-7945-A3FE-EC48E23980DB}">
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -3214,6 +3318,210 @@
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
         <v>30</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="G102" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E103" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G103" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E104" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="G104" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E105" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G105" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E106" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="G106" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E107" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G107" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E108" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="G108" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E109" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G109" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E110" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G110" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E111" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="G111" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E112" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G112" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="113" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E113" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G113" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="114" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E114" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="G114" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="115" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E115" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="G115" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="116" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E116" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="G116" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="117" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E117" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G117" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="118" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E118" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="G118" t="s">
+        <v>69</v>
+      </c>
+      <c r="H118" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="119" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E119" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G119" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="120" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E120" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G120" t="s">
+        <v>69</v>
+      </c>
+      <c r="H120" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="121" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E121" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="G121" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="122" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E122" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="G122" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="123" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E123" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="G123" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="124" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E124" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G124" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="125" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E125" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="G125" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="126" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E126" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="G126" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
draft1 vertical flow. card data not finished
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6388662F-BCFE-174B-B3C5-1324176A13C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C279EB-5FE2-EC48-9636-75BC34B5422F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
+    <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Faser" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="413">
   <si>
     <t>phase_id</t>
   </si>
@@ -198,9 +198,6 @@
   </si>
   <si>
     <t>Kollatering</t>
-  </si>
-  <si>
-    <t>Repetitioner</t>
   </si>
   <si>
     <t>2 månader</t>
@@ -1032,12 +1029,321 @@
 Kostym
 Övriga vid behov</t>
   </si>
+  <si>
+    <t>Ansvarig producent sammankallar
+Inspicienten kartlägger behoven för kollationeringen
+Inspicienten koordinerar med de olika tekniska avdelningarna för att verkställa repetitionen</t>
+  </si>
+  <si>
+    <t>Repetitioner 1</t>
+  </si>
+  <si>
+    <t>task-101</t>
+  </si>
+  <si>
+    <t>task-102</t>
+  </si>
+  <si>
+    <t>task-103</t>
+  </si>
+  <si>
+    <t>task-104</t>
+  </si>
+  <si>
+    <t>task-105</t>
+  </si>
+  <si>
+    <t>task-106</t>
+  </si>
+  <si>
+    <t>task-107</t>
+  </si>
+  <si>
+    <t>task-108</t>
+  </si>
+  <si>
+    <t>task-109</t>
+  </si>
+  <si>
+    <t>task-110</t>
+  </si>
+  <si>
+    <t>task-111</t>
+  </si>
+  <si>
+    <t>task-112</t>
+  </si>
+  <si>
+    <t>task-113</t>
+  </si>
+  <si>
+    <t>task-114</t>
+  </si>
+  <si>
+    <t>task-115</t>
+  </si>
+  <si>
+    <t>task-116</t>
+  </si>
+  <si>
+    <t>task-117</t>
+  </si>
+  <si>
+    <t>task-118</t>
+  </si>
+  <si>
+    <t>task-119</t>
+  </si>
+  <si>
+    <t>task-120</t>
+  </si>
+  <si>
+    <t>task-121</t>
+  </si>
+  <si>
+    <t>task-122</t>
+  </si>
+  <si>
+    <t>task-123</t>
+  </si>
+  <si>
+    <t>task-124</t>
+  </si>
+  <si>
+    <t>task-125</t>
+  </si>
+  <si>
+    <t>Kostymprovningar</t>
+  </si>
+  <si>
+    <t>Provmask</t>
+  </si>
+  <si>
+    <t>Sista 3D-scanningar</t>
+  </si>
+  <si>
+    <t>Påklädare / Maskmöte</t>
+  </si>
+  <si>
+    <t>Planering av tekniska dagar</t>
+  </si>
+  <si>
+    <t>Inbjudningslista godkända</t>
+  </si>
+  <si>
+    <t>Beslut om programblad</t>
+  </si>
+  <si>
+    <t>task-126</t>
+  </si>
+  <si>
+    <t>task-127</t>
+  </si>
+  <si>
+    <t>task-128</t>
+  </si>
+  <si>
+    <t>task-129</t>
+  </si>
+  <si>
+    <t>task-130</t>
+  </si>
+  <si>
+    <t>task-131</t>
+  </si>
+  <si>
+    <t>task-132</t>
+  </si>
+  <si>
+    <t>task-133</t>
+  </si>
+  <si>
+    <t>task-134</t>
+  </si>
+  <si>
+    <t>Ansvarig producent definierar tidsram
+Teknisk chef övervakar
+Tekniska planeraren samt scenmästaren ansvarar för att scenografin monteras innan repetitionsstart på scen
+Samtliga scenografielement färdiga tills de tekniska dagarna
+Ljus- opch ljudbygge</t>
+  </si>
+  <si>
+    <t>task-135</t>
+  </si>
+  <si>
+    <t>task-136</t>
+  </si>
+  <si>
+    <t>task-137</t>
+  </si>
+  <si>
+    <t>task-138</t>
+  </si>
+  <si>
+    <t>task-139</t>
+  </si>
+  <si>
+    <t>task-140</t>
+  </si>
+  <si>
+    <t>task-141</t>
+  </si>
+  <si>
+    <t>task-142</t>
+  </si>
+  <si>
+    <t>task-143</t>
+  </si>
+  <si>
+    <t>task-144</t>
+  </si>
+  <si>
+    <t>task-145</t>
+  </si>
+  <si>
+    <t>task-146</t>
+  </si>
+  <si>
+    <t>task-147</t>
+  </si>
+  <si>
+    <t>Genomgång av scenbilder och -byten</t>
+  </si>
+  <si>
+    <t>Scenografins finjusteringar på scenen</t>
+  </si>
+  <si>
+    <t>Säkerhetsgenomgång</t>
+  </si>
+  <si>
+    <t>Säkerhetsgranskning</t>
+  </si>
+  <si>
+    <t>Kostym- och maskkorigeringar</t>
+  </si>
+  <si>
+    <t>Påklädare &amp; Maskmöte nr. 2</t>
+  </si>
+  <si>
+    <t>Sitzprobe</t>
+  </si>
+  <si>
+    <t>Tekniska repetitioner med ensemble</t>
+  </si>
+  <si>
+    <t>Inkörning av tekniska turare</t>
+  </si>
+  <si>
+    <t>Premiär</t>
+  </si>
+  <si>
+    <t>Orkester rep.</t>
+  </si>
+  <si>
+    <t>Förberedande generalrepetitioner (ÖVERFLÖDIG?)</t>
+  </si>
+  <si>
+    <t>Genrep 1-3</t>
+  </si>
+  <si>
+    <t>Förberedande genrep 1-3</t>
+  </si>
+  <si>
+    <t>task-148</t>
+  </si>
+  <si>
+    <t>Manus (process)</t>
+  </si>
+  <si>
+    <t>Textning klar</t>
+  </si>
+  <si>
+    <t>Fotograferingar</t>
+  </si>
+  <si>
+    <t>Provpublik</t>
+  </si>
+  <si>
+    <t>task-149</t>
+  </si>
+  <si>
+    <t>task-150</t>
+  </si>
+  <si>
+    <t>task-151</t>
+  </si>
+  <si>
+    <t>task-152</t>
+  </si>
+  <si>
+    <t>US-repetitioner</t>
+  </si>
+  <si>
+    <t>Sista föreställningen</t>
+  </si>
+  <si>
+    <t>Inkörning av tekniska turare 2 veckor efter premiär</t>
+  </si>
+  <si>
+    <t>Feedback</t>
+  </si>
+  <si>
+    <t>Teosto-rapportering</t>
+  </si>
+  <si>
+    <t>Rivning, scenografi</t>
+  </si>
+  <si>
+    <t>Rivning, ljus</t>
+  </si>
+  <si>
+    <t>task-153</t>
+  </si>
+  <si>
+    <t>task-154</t>
+  </si>
+  <si>
+    <t>task-155</t>
+  </si>
+  <si>
+    <t>task-156</t>
+  </si>
+  <si>
+    <t>task-157</t>
+  </si>
+  <si>
+    <t>task-158</t>
+  </si>
+  <si>
+    <t>task-159</t>
+  </si>
+  <si>
+    <t>task-160</t>
+  </si>
+  <si>
+    <t>Rivning, ateljé</t>
+  </si>
+  <si>
+    <t>taas-155</t>
+  </si>
+  <si>
+    <t>Ekonomirapportering</t>
+  </si>
+  <si>
+    <t>Publikstatistik</t>
+  </si>
+  <si>
+    <t>Royaltyberäkningar</t>
+  </si>
+  <si>
+    <t>Arkivering</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1065,6 +1371,12 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1086,7 +1398,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1099,6 +1411,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1451,10 +1764,10 @@
         <v>20</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>1</v>
@@ -1557,7 +1870,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="204" x14ac:dyDescent="0.2">
@@ -1577,7 +1890,7 @@
         <v>46</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="136" x14ac:dyDescent="0.2">
@@ -1597,10 +1910,10 @@
         <v>47</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1611,35 +1924,41 @@
         <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G9" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="136" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C10" t="s">
         <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>52</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
         <v>33</v>
@@ -1648,15 +1967,15 @@
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1667,7 +1986,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D990BC4-CB70-7945-A3FE-EC48E23980DB}">
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -1686,19 +2005,19 @@
         <v>12</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="340" x14ac:dyDescent="0.2">
@@ -1712,10 +2031,10 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="G2" t="s">
         <v>16</v>
@@ -1729,10 +2048,10 @@
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G3" t="s">
         <v>16</v>
@@ -1746,10 +2065,10 @@
         <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G4" t="s">
         <v>16</v>
@@ -1757,16 +2076,16 @@
     </row>
     <row r="5" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
         <v>16</v>
@@ -1774,13 +2093,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G6" t="s">
         <v>16</v>
@@ -1788,13 +2107,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G7" t="s">
         <v>16</v>
@@ -1802,13 +2121,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G8" t="s">
         <v>16</v>
@@ -1816,262 +2135,262 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
         <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
         <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B19" t="s">
         <v>25</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B20" t="s">
         <v>25</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
         <v>25</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B22" t="s">
         <v>25</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B24" t="s">
         <v>25</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B25" t="s">
         <v>25</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B26" t="s">
         <v>25</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="136" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B27" t="s">
         <v>25</v>
@@ -2080,18 +2399,18 @@
         <v>18</v>
       </c>
       <c r="E27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="G27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B28" t="s">
         <v>25</v>
@@ -2100,15 +2419,15 @@
         <v>18</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B29" t="s">
         <v>25</v>
@@ -2117,15 +2436,15 @@
         <v>18</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" t="s">
         <v>25</v>
@@ -2134,15 +2453,15 @@
         <v>18</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B31" t="s">
         <v>25</v>
@@ -2151,15 +2470,15 @@
         <v>18</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B32" t="s">
         <v>25</v>
@@ -2168,15 +2487,15 @@
         <v>18</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B33" t="s">
         <v>25</v>
@@ -2185,15 +2504,15 @@
         <v>18</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B34" t="s">
         <v>25</v>
@@ -2202,15 +2521,15 @@
         <v>18</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B35" t="s">
         <v>25</v>
@@ -2219,15 +2538,15 @@
         <v>18</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
         <v>25</v>
@@ -2236,15 +2555,15 @@
         <v>18</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B37" t="s">
         <v>25</v>
@@ -2253,141 +2572,141 @@
         <v>18</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B38" t="s">
         <v>26</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B39" t="s">
         <v>26</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B40" t="s">
         <v>26</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B41" t="s">
         <v>26</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B42" t="s">
         <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B43" t="s">
         <v>26</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B44" t="s">
         <v>26</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B45" t="s">
         <v>26</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G45" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B46" t="s">
         <v>26</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B47" t="s">
         <v>27</v>
@@ -2396,18 +2715,18 @@
         <v>10</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G47" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H47" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B48" t="s">
         <v>27</v>
@@ -2416,18 +2735,18 @@
         <v>10</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H48" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B49" t="s">
         <v>27</v>
@@ -2436,19 +2755,19 @@
         <v>10</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H49" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B50" t="s">
         <v>27</v>
@@ -2457,18 +2776,18 @@
         <v>10</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G50" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H50" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B51" t="s">
         <v>27</v>
@@ -2477,18 +2796,18 @@
         <v>10</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G51" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H51" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B52" t="s">
         <v>27</v>
@@ -2497,18 +2816,18 @@
         <v>10</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G52" t="s">
+        <v>61</v>
+      </c>
+      <c r="H52" t="s">
         <v>180</v>
-      </c>
-      <c r="G52" t="s">
-        <v>62</v>
-      </c>
-      <c r="H52" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
@@ -2517,18 +2836,18 @@
         <v>10</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H53" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -2537,18 +2856,18 @@
         <v>10</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G54" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H54" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B55" t="s">
         <v>27</v>
@@ -2557,18 +2876,18 @@
         <v>10</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G55" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B56" t="s">
         <v>27</v>
@@ -2577,18 +2896,18 @@
         <v>10</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B57" t="s">
         <v>27</v>
@@ -2597,18 +2916,18 @@
         <v>10</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H57" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B58" t="s">
         <v>27</v>
@@ -2617,18 +2936,18 @@
         <v>10</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G58" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H58" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B59" t="s">
         <v>27</v>
@@ -2637,18 +2956,18 @@
         <v>10</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H59" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B60" t="s">
         <v>27</v>
@@ -2657,18 +2976,18 @@
         <v>10</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H60" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B61" t="s">
         <v>27</v>
@@ -2677,18 +2996,18 @@
         <v>10</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H61" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B62" t="s">
         <v>27</v>
@@ -2697,831 +3016,1526 @@
         <v>10</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H62" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
       </c>
       <c r="C63" t="s">
+        <v>206</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="G63" t="s">
+        <v>60</v>
+      </c>
+      <c r="H63" t="s">
         <v>207</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G63" t="s">
-        <v>61</v>
-      </c>
-      <c r="H63" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B64" t="s">
         <v>27</v>
       </c>
       <c r="C64" t="s">
+        <v>206</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G64" t="s">
+        <v>60</v>
+      </c>
+      <c r="H64" t="s">
         <v>207</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G64" t="s">
-        <v>61</v>
-      </c>
-      <c r="H64" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B65" t="s">
         <v>27</v>
       </c>
       <c r="C65" t="s">
+        <v>206</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G65" t="s">
+        <v>60</v>
+      </c>
+      <c r="H65" t="s">
         <v>207</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="G65" t="s">
-        <v>61</v>
-      </c>
-      <c r="H65" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B66" t="s">
         <v>27</v>
       </c>
       <c r="C66" t="s">
+        <v>206</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G66" t="s">
+        <v>60</v>
+      </c>
+      <c r="H66" t="s">
         <v>207</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G66" t="s">
-        <v>61</v>
-      </c>
-      <c r="H66" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B67" t="s">
         <v>27</v>
       </c>
       <c r="C67" t="s">
+        <v>206</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G67" t="s">
+        <v>60</v>
+      </c>
+      <c r="H67" t="s">
         <v>207</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="G67" t="s">
-        <v>61</v>
-      </c>
-      <c r="H67" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B68" t="s">
         <v>27</v>
       </c>
       <c r="C68" t="s">
+        <v>206</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G68" t="s">
+        <v>60</v>
+      </c>
+      <c r="H68" t="s">
         <v>207</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G68" t="s">
-        <v>61</v>
-      </c>
-      <c r="H68" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B69" t="s">
         <v>27</v>
       </c>
       <c r="C69" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G69" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H69" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B70" t="s">
         <v>27</v>
       </c>
       <c r="C70" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G70" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H70" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B71" t="s">
         <v>27</v>
       </c>
       <c r="C71" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G71" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H71" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B72" t="s">
         <v>28</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G72" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B73" t="s">
         <v>28</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G73" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B74" t="s">
         <v>28</v>
       </c>
       <c r="D74" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G74" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B75" t="s">
         <v>28</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G75" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B76" t="s">
         <v>28</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B77" t="s">
         <v>28</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G77" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B78" t="s">
         <v>28</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G78" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B79" t="s">
         <v>28</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G79" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B80" t="s">
         <v>28</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G80" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B81" t="s">
         <v>28</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G81" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B82" t="s">
         <v>28</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G82" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B83" t="s">
         <v>28</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G83" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B84" t="s">
         <v>29</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G84" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B85" t="s">
         <v>29</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G85" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H85" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B86" t="s">
         <v>29</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G86" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B87" t="s">
         <v>29</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G87" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B88" t="s">
         <v>29</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G88" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B89" t="s">
         <v>29</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G89" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B90" t="s">
         <v>29</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G90" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B91" t="s">
         <v>29</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B92" t="s">
         <v>29</v>
       </c>
       <c r="E92" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G92" t="s">
+        <v>70</v>
+      </c>
+      <c r="H92" t="s">
         <v>253</v>
-      </c>
-      <c r="G92" t="s">
-        <v>71</v>
-      </c>
-      <c r="H92" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B93" t="s">
         <v>29</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G93" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B94" t="s">
         <v>29</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G94" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B95" t="s">
         <v>29</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G95" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B96" t="s">
         <v>29</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G96" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B97" t="s">
         <v>29</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G97" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B98" t="s">
         <v>29</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G98" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B99" t="s">
         <v>29</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G99" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B100" t="s">
         <v>29</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G100" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B101" t="s">
         <v>29</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G101" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>314</v>
+      </c>
       <c r="B102" t="s">
         <v>30</v>
       </c>
       <c r="E102" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G102" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>315</v>
+      </c>
+      <c r="B103" t="s">
+        <v>30</v>
+      </c>
+      <c r="E103" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="G102" t="s">
+      <c r="G103" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>316</v>
+      </c>
+      <c r="B104" t="s">
+        <v>30</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G104" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>317</v>
+      </c>
+      <c r="B105" t="s">
+        <v>30</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="G105" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>318</v>
+      </c>
+      <c r="B106" t="s">
+        <v>30</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G106" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>319</v>
+      </c>
+      <c r="B107" t="s">
+        <v>30</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="G107" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>320</v>
+      </c>
+      <c r="B108" t="s">
+        <v>30</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G108" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>321</v>
+      </c>
+      <c r="B109" t="s">
+        <v>30</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G109" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>322</v>
+      </c>
+      <c r="B110" t="s">
+        <v>30</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="G110" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>323</v>
+      </c>
+      <c r="B111" t="s">
+        <v>30</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G111" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E103" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="G103" t="s">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>324</v>
+      </c>
+      <c r="B112" t="s">
+        <v>30</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="G112" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E104" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="G104" t="s">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>325</v>
+      </c>
+      <c r="B113" t="s">
+        <v>30</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G113" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>326</v>
+      </c>
+      <c r="B114" t="s">
+        <v>30</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G114" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>327</v>
+      </c>
+      <c r="B115" t="s">
+        <v>30</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="G115" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>328</v>
+      </c>
+      <c r="B116" t="s">
+        <v>30</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="G116" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>329</v>
+      </c>
+      <c r="B117" t="s">
+        <v>30</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="G117" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>330</v>
+      </c>
+      <c r="B118" t="s">
+        <v>30</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G118" t="s">
+        <v>68</v>
+      </c>
+      <c r="H118" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>331</v>
+      </c>
+      <c r="B119" t="s">
+        <v>30</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="G119" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>332</v>
+      </c>
+      <c r="B120" t="s">
+        <v>30</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G120" t="s">
+        <v>68</v>
+      </c>
+      <c r="H120" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>333</v>
+      </c>
+      <c r="B121" t="s">
+        <v>30</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G121" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>334</v>
+      </c>
+      <c r="B122" t="s">
+        <v>30</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="G122" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>335</v>
+      </c>
+      <c r="B123" t="s">
+        <v>30</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="G123" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>336</v>
+      </c>
+      <c r="B124" t="s">
+        <v>30</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="G124" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>337</v>
+      </c>
+      <c r="B125" t="s">
+        <v>30</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G125" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>338</v>
+      </c>
+      <c r="B126" t="s">
+        <v>30</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="G126" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>346</v>
+      </c>
+      <c r="B127" t="s">
+        <v>31</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="G127" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>347</v>
+      </c>
+      <c r="B128" t="s">
+        <v>31</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="G128" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>348</v>
+      </c>
+      <c r="B129" t="s">
+        <v>31</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G129" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>349</v>
+      </c>
+      <c r="B130" t="s">
+        <v>31</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="G130" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>350</v>
+      </c>
+      <c r="B131" t="s">
+        <v>31</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="G131" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>351</v>
+      </c>
+      <c r="B132" t="s">
+        <v>31</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G132" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>352</v>
+      </c>
+      <c r="B133" t="s">
+        <v>31</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G133" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>353</v>
+      </c>
+      <c r="B134" t="s">
+        <v>31</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="G134" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
+        <v>354</v>
+      </c>
+      <c r="B135" t="s">
+        <v>31</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="G135" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>356</v>
+      </c>
+      <c r="B136" t="s">
+        <v>53</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G136" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
+        <v>357</v>
+      </c>
+      <c r="B137" t="s">
+        <v>53</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="G137" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>358</v>
+      </c>
+      <c r="B138" t="s">
+        <v>53</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G138" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
+        <v>359</v>
+      </c>
+      <c r="B139" t="s">
+        <v>53</v>
+      </c>
+      <c r="D139" t="s">
+        <v>358</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G139" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>360</v>
+      </c>
+      <c r="B140" t="s">
+        <v>53</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="G140" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
+        <v>361</v>
+      </c>
+      <c r="B141" t="s">
+        <v>53</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="G141" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
+        <v>362</v>
+      </c>
+      <c r="B142" t="s">
+        <v>53</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="G142" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E105" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="G105" t="s">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>363</v>
+      </c>
+      <c r="B143" t="s">
+        <v>53</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="G143" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E106" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="G106" t="s">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>364</v>
+      </c>
+      <c r="B144" t="s">
+        <v>53</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="G144" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E107" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="G107" t="s">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>365</v>
+      </c>
+      <c r="B145" t="s">
+        <v>53</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G145" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>366</v>
+      </c>
+      <c r="B146" t="s">
+        <v>53</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="G146" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
+        <v>367</v>
+      </c>
+      <c r="B147" t="s">
+        <v>53</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="G147" t="s">
+        <v>68</v>
+      </c>
+      <c r="H147" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
+        <v>368</v>
+      </c>
+      <c r="B148" t="s">
+        <v>53</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="G148" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
+        <v>383</v>
+      </c>
+      <c r="B149" t="s">
+        <v>53</v>
+      </c>
+      <c r="D149" t="s">
+        <v>368</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="G149" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>388</v>
+      </c>
+      <c r="B150" t="s">
+        <v>53</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="G150" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>389</v>
+      </c>
+      <c r="B151" t="s">
+        <v>53</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="G151" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>390</v>
+      </c>
+      <c r="B152" t="s">
+        <v>53</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="G152" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>391</v>
+      </c>
+      <c r="B153" t="s">
+        <v>53</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G153" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
+        <v>399</v>
+      </c>
+      <c r="B154" t="s">
+        <v>54</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G154" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>400</v>
+      </c>
+      <c r="B155" t="s">
+        <v>54</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="G155" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>401</v>
+      </c>
+      <c r="B156" t="s">
+        <v>54</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="G156" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
+        <v>402</v>
+      </c>
+      <c r="B157" t="s">
+        <v>54</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="G157" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E108" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="G108" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E109" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G109" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E110" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="G110" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E111" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="G111" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E112" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="G112" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="113" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E113" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G113" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="114" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E114" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="G114" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="115" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E115" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="G115" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="116" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E116" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="G116" t="s">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
+        <v>403</v>
+      </c>
+      <c r="B158" t="s">
+        <v>54</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G158" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
+        <v>404</v>
+      </c>
+      <c r="B159" t="s">
+        <v>54</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G159" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
+        <v>405</v>
+      </c>
+      <c r="B160" t="s">
+        <v>54</v>
+      </c>
+      <c r="D160" t="s">
+        <v>401</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="G160" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
+        <v>406</v>
+      </c>
+      <c r="B161" t="s">
+        <v>54</v>
+      </c>
+      <c r="D161" t="s">
+        <v>401</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G161" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D162" t="s">
+        <v>408</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="G162" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E163" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="G163" s="6" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="117" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E117" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="G117" t="s">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E164" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G164" s="6" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="118" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E118" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="G118" t="s">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E165" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="G165" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="H118" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="119" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E119" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="G119" t="s">
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E166" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G166" s="6" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="120" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E120" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="G120" t="s">
-        <v>69</v>
-      </c>
-      <c r="H120" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="121" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E121" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="G121" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="122" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E122" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="G122" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="123" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E123" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="G123" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="124" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E124" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="G124" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="125" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E125" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="G125" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="126" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E126" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="G126" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -3549,10 +4563,10 @@
         <v>7</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="119" x14ac:dyDescent="0.2">
@@ -3563,10 +4577,10 @@
         <v>25</v>
       </c>
       <c r="C2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -3577,10 +4591,10 @@
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -3591,7 +4605,7 @@
         <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -3610,47 +4624,47 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
         <v>67</v>
-      </c>
-      <c r="B5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
@@ -3658,26 +4672,26 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
draft1, gantt task filter feature
</commit_message>
<xml_diff>
--- a/st-process.xlsx
+++ b/st-process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julius/dev/svenska-teatern/produktionsprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C279EB-5FE2-EC48-9636-75BC34B5422F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51D5FD3-5578-8F48-8BF9-7D9D51F11BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60160" yWindow="-15340" windowWidth="30080" windowHeight="33340" activeTab="1" xr2:uid="{873CCD51-E24D-F745-888B-A4D006586D0A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="417">
   <si>
     <t>phase_id</t>
   </si>
@@ -1324,9 +1324,6 @@
     <t>Rivning, ateljé</t>
   </si>
   <si>
-    <t>taas-155</t>
-  </si>
-  <si>
     <t>Ekonomirapportering</t>
   </si>
   <si>
@@ -1337,6 +1334,21 @@
   </si>
   <si>
     <t>Arkivering</t>
+  </si>
+  <si>
+    <t>task-161</t>
+  </si>
+  <si>
+    <t>task-162</t>
+  </si>
+  <si>
+    <t>task-163</t>
+  </si>
+  <si>
+    <t>task-164</t>
+  </si>
+  <si>
+    <t>task-165</t>
   </si>
 </sst>
 </file>
@@ -4496,8 +4508,14 @@
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
+        <v>412</v>
+      </c>
+      <c r="B162" t="s">
+        <v>54</v>
+      </c>
       <c r="D162" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>407</v>
@@ -4507,32 +4525,56 @@
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
+        <v>413</v>
+      </c>
+      <c r="B163" t="s">
+        <v>54</v>
+      </c>
       <c r="E163" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G163" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
+        <v>414</v>
+      </c>
+      <c r="B164" t="s">
+        <v>54</v>
+      </c>
       <c r="E164" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="G164" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
+        <v>415</v>
+      </c>
+      <c r="B165" t="s">
+        <v>54</v>
+      </c>
       <c r="E165" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G165" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
+        <v>416</v>
+      </c>
+      <c r="B166" t="s">
+        <v>54</v>
+      </c>
       <c r="E166" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G166" s="6" t="s">
         <v>69</v>

</xml_diff>